<commit_message>
Référentiel ESR : une école d'ingénieurs compte pour un établissement (écoles internes, écoles de l'IMT) — 2.23.0
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xs9aCmvKzLyadh5owJLUJw
</commit_message>
<xml_diff>
--- a/tests/donnees/referentiel_esr_essai.xlsx
+++ b/tests/donnees/referentiel_esr_essai.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1034,6 +1034,421 @@
       <c r="Y6" t="inlineStr">
         <is>
           <t>Campus de Saint-Malo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ETAB-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>École supérieure d'ingénieurs de Rennes (ESIR)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ESIR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>École supérieure d'ingénieurs de Rennes</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ESIR</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Composante interne</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>École d'ingénieurs interne</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ETAB-0001 – Université de Rennes</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0352480F</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>CTI</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Existante</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>École supérieure d'ingénieurs de Rennes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ETAB-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom (IMT)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IMT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom, au périmètre des écoles IMT Atlantique, Lille Douai, Albi, Alès, Mines Saint-Étienne et Institut Mines-Télécom Business school</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>IMT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Établissement</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Grand établissement</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Palaiseau</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0912424R</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>PLF</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Existante</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ETAB-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IMT Atlantique</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>IMT Atlantique</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>IMT Atlantique</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Composante interne</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>École d'ingénieurs interne</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>ETAB-0007 – Institut Mines-Télécom, au périmètre des écoles IMT Atlantique, Lille Douai, Albi, Alès, Mines Saint-Étienne et Institut Mines-Télécom Business school</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Brest</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0442852L</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>CTI</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Existante</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>IMT Atlantique</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ETAB-0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom Business School</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>IMT-BS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom Business School</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>IMT-BS</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Composante interne</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Autre composante interne</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>ETAB-0007 – Institut Mines-Télécom, au périmètre des écoles IMT Atlantique, Lille Douai, Albi, Alès, Mines Saint-Étienne et Institut Mines-Télécom Business school</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Versailles</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Évry-Courcouronnes</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0912255G</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Paysage</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Existante</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>IMT Business School</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ETAB-0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IMT Atlantique - Campus de Rennes</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>IMT Atlantique Rennes</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>IMT Atlantique - Campus de Rennes</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Site ou campus</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Campus ou site</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>ETAB-0007 – Institut Mines-Télécom, au périmètre des écoles IMT Atlantique, Lille Douai, Albi, Alès, Mines Saint-Étienne et Institut Mines-Télécom Business school</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>public</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Cesson-Sévigné</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Paysage</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Ajoutée (Paysage) – à valider</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>IMT Atlantique - Campus de Rennes</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1090,6 +1505,41 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>Campus de Saint-Malo – Université Rennes 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>École supérieure d'ingénieurs de Rennes (ESIR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom (IMT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IMT Atlantique</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom Business School</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IMT Atlantique - Campus de Rennes</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1647,6 +2097,142 @@
       </c>
       <c r="S7" t="n">
         <v>9000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SITE-0008</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ETAB-0001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Université de Rennes</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ETAB-0006 – École supérieure d'ingénieurs de Rennes</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ESIR Beaulieu</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>OAD</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>35042</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>263 av. Leclerc</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>48.1172</v>
+      </c>
+      <c r="O8" t="n">
+        <v>-1.638</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Source du site</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SITE-0009</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ETAB-0007</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Institut Mines-Télécom</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ETAB-0008 – IMT Atlantique</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Campus de Brest</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Validé</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>OAD</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Plouzané</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>29280</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Technopôle Brest-Iroise</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>48.359</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-4.57</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Source du site</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>